<commit_message>
docs(tracker): update Master Backlog Status to live reality; workbook is the authoritative current tracker again
Status column was a 24-Jun planning snapshot (completed items still showed OPEN). Updated 30-Jun: 19 DONE, 1 PARTIAL, 16 BLOCKED (founder/credential), 1 DECISION, 1 FOUNDER, 13 OPEN (future modules), 1 N/A. Tracker doc only - no code/feature changes.
</commit_message>
<xml_diff>
--- a/Review/RKM_FOUNDATION_MASTER_BUILD_WORKBOOK_V2.1.xlsx
+++ b/Review/RKM_FOUNDATION_MASTER_BUILD_WORKBOOK_V2.1.xlsx
@@ -1374,7 +1374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>DONE - live</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>DONE - live</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>DONE - live</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DONE - live</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>BLOCKED - provider live; 28-day baseline needs Plausible acct + time</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1785,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>DONE - live</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>DONE - live</t>
         </is>
       </c>
     </row>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="K9" s="9" t="inlineStr">
         <is>
-          <t>IN-PR</t>
+          <t>DONE - junk purged + .gitignore</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>DONE - live</t>
         </is>
       </c>
     </row>
@@ -2013,7 +2013,7 @@
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>FACT-BLOCKED</t>
+          <t>DONE - live 30-Jun (95/5 commitment strip at the ask)</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>FACT-BLOCKED</t>
+          <t>PARTIAL - 3 tiers + custom live; 4th low tier/cost refinement pending (see 014)</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>FACT-BLOCKED</t>
+          <t>BLOCKED - founder: no impact numbers yet (intentionally omitted)</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>N/A - UPI rejected by Razorpay; removed from UI 29-Jun</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DECISION - founder: lower floor Rs.1000 -&gt; Rs.500? pending</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>BLOCKED - needs analytics(005) + donor data</t>
         </is>
       </c>
     </row>
@@ -2355,7 +2355,7 @@
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>FACT-BLOCKED</t>
+          <t>BLOCKED - founder: audited financials (95/5 commitment shipped as interim)</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2412,7 @@
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>FACT-BLOCKED</t>
+          <t>BLOCKED - founder: leadership names/photos/consent</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>FACT-BLOCKED</t>
+          <t>BLOCKED - founder: third-party validation data</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>FACT-BLOCKED</t>
+          <t>BLOCKED - founder: real named stories + photos (placeholder live)</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DONE - live (Tobler home story)</t>
         </is>
       </c>
     </row>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>BUILD-BLOCKED</t>
+          <t>DONE - live (self-host fonts)</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DONE - live (next/image)</t>
         </is>
       </c>
     </row>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DONE - live (nonce CSP)</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DONE - donation E2E in CI</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DONE - manual WCAG 2.2 AA pass</t>
         </is>
       </c>
     </row>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DONE - reduced-motion verified</t>
         </is>
       </c>
     </row>
@@ -2982,7 +2982,7 @@
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DONE - prototype routes noindexed (robots.ts)</t>
         </is>
       </c>
     </row>
@@ -3039,7 +3039,7 @@
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - commit DB migrations (needs schema export)</t>
         </is>
       </c>
     </row>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - per-user admin auth (future module)</t>
         </is>
       </c>
     </row>
@@ -3153,7 +3153,7 @@
       </c>
       <c r="K31" s="10" t="inlineStr">
         <is>
-          <t>FOUNDER</t>
+          <t>FOUNDER - rotate exposed secrets</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>DATA-BLOCKED</t>
+          <t>BLOCKED - donor data</t>
         </is>
       </c>
     </row>
@@ -3267,7 +3267,7 @@
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - CSR landing rebuild</t>
         </is>
       </c>
     </row>
@@ -3324,7 +3324,7 @@
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>FACT-BLOCKED</t>
+          <t>BLOCKED - founder: CSR case studies</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>DATA-BLOCKED</t>
+          <t>BLOCKED - donor data</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3438,7 @@
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DONE (skeleton) - branch; live-send blocked on RESEND key + content</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3495,7 @@
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>DATA-BLOCKED</t>
+          <t>BLOCKED - donor data (win-back skeleton exists)</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>FACT-BLOCKED</t>
+          <t>BLOCKED - founder: impact numbers (skeleton exists)</t>
         </is>
       </c>
     </row>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - WhatsApp journeys (future module)</t>
         </is>
       </c>
     </row>
@@ -3666,7 +3666,7 @@
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - campaign calendar (future)</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>BLOCKED - founder: named animals (Guardian/Sponsor program)</t>
         </is>
       </c>
     </row>
@@ -3780,7 +3780,7 @@
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - volunteer-&gt;donor path (future module)</t>
         </is>
       </c>
     </row>
@@ -3837,7 +3837,7 @@
       </c>
       <c r="K43" s="6" t="inlineStr">
         <is>
-          <t>FACT-BLOCKED</t>
+          <t>DONE - no FCRA; site states INR/domestic-only</t>
         </is>
       </c>
     </row>
@@ -3894,7 +3894,7 @@
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - EN/HI shared content model (future refactor)</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - legacy/wills page (needs legal wording)</t>
         </is>
       </c>
     </row>
@@ -4008,7 +4008,7 @@
       </c>
       <c r="K46" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - tribute/memorial giving (future module)</t>
         </is>
       </c>
     </row>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="K47" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - P2P /fundraiser optimisation (future)</t>
         </is>
       </c>
     </row>
@@ -4122,7 +4122,7 @@
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>FACT-BLOCKED</t>
+          <t>BLOCKED - founder: real adoptable animals</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4179,7 @@
       </c>
       <c r="K49" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>BLOCKED - founder: supply/wishlist</t>
         </is>
       </c>
     </row>
@@ -4236,7 +4236,7 @@
       </c>
       <c r="K50" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - shop funnel audit</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="K51" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - content/SEO plan (marketing)</t>
         </is>
       </c>
     </row>
@@ -4350,7 +4350,7 @@
       </c>
       <c r="K52" s="6" t="inlineStr">
         <is>
-          <t>DATA-BLOCKED</t>
+          <t>BLOCKED - needs real-device + field traffic (005)</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,14 @@
       </c>
       <c r="K53" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - email deliverability (needs RESEND send)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Status column updated 30 Jun 2026 to reflect live execution state (prior values were the 24 Jun planning snapshot).</t>
         </is>
       </c>
     </row>

</xml_diff>